<commit_message>
create two new test (product list pieces check, product list names test)
</commit_message>
<xml_diff>
--- a/docs/requirement-table.xlsx
+++ b/docs/requirement-table.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t xml:space="preserve">Vizsgaremek követelményeinek megfelelés</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t xml:space="preserve">Adatok listázása</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC05 , TC06</t>
   </si>
   <si>
     <t xml:space="preserve">Több oldalas lista bejárás</t>
@@ -391,46 +394,49 @@
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="B7" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
create new test (registerMultipleUsersFromCsv)
</commit_message>
<xml_diff>
--- a/docs/requirement-table.xlsx
+++ b/docs/requirement-table.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t xml:space="preserve">Vizsgaremek követelményeinek megfelelés</t>
   </si>
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Regisztráció</t>
   </si>
   <si>
-    <t xml:space="preserve">TC01 , TC02 </t>
+    <t xml:space="preserve">TC01 , TC02 , TC09</t>
   </si>
   <si>
     <t xml:space="preserve">Pozitív és negatív teszt </t>
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Bejelentkezés</t>
   </si>
   <si>
-    <t xml:space="preserve">TC03</t>
+    <t xml:space="preserve">TC03 , TC09</t>
   </si>
   <si>
     <t xml:space="preserve">Adatkezelési nyilatkozat használata </t>
@@ -73,13 +73,16 @@
     <t xml:space="preserve">Új adat bevitel </t>
   </si>
   <si>
-    <t xml:space="preserve">TC01 , TC08</t>
+    <t xml:space="preserve">TC01 , TC08 , TC09 </t>
   </si>
   <si>
     <t xml:space="preserve">TC08 fájlfeltöltéssel</t>
   </si>
   <si>
     <t xml:space="preserve">Ismételt és sorozatos adatbevitel adatforrásból</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC09</t>
   </si>
   <si>
     <t xml:space="preserve">Meglévő adat módosítás	</t>
@@ -430,25 +433,28 @@
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="B10" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
almost finish addProductChangeQuantityViaReadAndRemove test
</commit_message>
<xml_diff>
--- a/docs/requirement-table.xlsx
+++ b/docs/requirement-table.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t xml:space="preserve">Vizsgaremek követelményeinek megfelelés</t>
   </si>
@@ -86,6 +86,9 @@
   </si>
   <si>
     <t xml:space="preserve">Meglévő adat módosítás	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC10</t>
   </si>
   <si>
     <t xml:space="preserve">Adat vagy adatok törlése </t>
@@ -441,20 +444,26 @@
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="B11" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
start to write ExportProductNameAndTheirPrices test
</commit_message>
<xml_diff>
--- a/docs/requirement-table.xlsx
+++ b/docs/requirement-table.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t xml:space="preserve">Vizsgaremek követelményeinek megfelelés</t>
   </si>
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Bejelentkezés</t>
   </si>
   <si>
-    <t xml:space="preserve">TC03 , TC09</t>
+    <t xml:space="preserve">TC01 , TC03 , TC09</t>
   </si>
   <si>
     <t xml:space="preserve">Adatkezelési nyilatkozat használata </t>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t xml:space="preserve">Adat vagy adatok törlése </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC01 , TC09</t>
   </si>
   <si>
     <t xml:space="preserve">Adatok lementése felületről</t>
@@ -452,18 +455,21 @@
       <c r="A12" s="1" t="s">
         <v>23</v>
       </c>
+      <c r="B12" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore: modify TC10 test case description and add to reqirement-table.xlsx
</commit_message>
<xml_diff>
--- a/docs/requirement-table.xlsx
+++ b/docs/requirement-table.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t xml:space="preserve">Vizsgaremek követelményeinek megfelelés</t>
   </si>
@@ -463,6 +463,9 @@
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="B13" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">

</xml_diff>

<commit_message>
chore: add @DisplayName and modify manual-test-cases file
</commit_message>
<xml_diff>
--- a/docs/requirement-table.xlsx
+++ b/docs/requirement-table.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t xml:space="preserve">Vizsgaremek követelményeinek megfelelés</t>
   </si>
@@ -98,6 +98,9 @@
   </si>
   <si>
     <t xml:space="preserve">Adatok lementése felületről</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC11</t>
   </si>
   <si>
     <t xml:space="preserve">Kijelentkezés</t>
@@ -464,12 +467,12 @@
         <v>25</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>24</v>

</xml_diff>